<commit_message>
docs: vincular entrega a la cuenta del curso
</commit_message>
<xml_diff>
--- a/SistemaInventarios/docs/Backlog.xlsx
+++ b/SistemaInventarios/docs/Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="1" r:id="R1be5fa44d8134a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="1" r:id="R797600634e344e1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
         <x:v>Terminado</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F6" s="8" t="str">
         <x:v>Abrir los formularios desde Inventario y volver al guardar o cancelar.</x:v>
@@ -404,7 +404,7 @@
         <x:v>Terminado</x:v>
       </x:c>
       <x:c r="E7" s="5" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F7" s="5" t="str">
         <x:v>Disponer de requisitos, Canvas, enlace Figma y esquema de categorías, productos y movimientos.</x:v>
@@ -424,7 +424,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E8" s="8" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F8" s="8" t="str">
         <x:v>Consultar productos por código o nombre y filtrar por categoría.</x:v>
@@ -444,7 +444,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F9" s="5" t="str">
         <x:v>Validar código único, campos requeridos y cantidades no negativas.</x:v>
@@ -464,7 +464,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E10" s="8" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F10" s="8" t="str">
         <x:v>Registrar movimiento y actualizar stock atómicamente; impedir stock negativo.</x:v>
@@ -484,7 +484,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
         <x:v>Marcar productos con stock actual menor al mínimo.</x:v>
@@ -504,7 +504,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E12" s="8" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F12" s="8" t="str">
         <x:v>Mostrar producto, tipo, cantidad, fecha y motivo de cada movimiento.</x:v>
@@ -524,7 +524,7 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>ricardoNP51</x:v>
+        <x:v>ricardoNP0</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str">
         <x:v>Verificar las reglas del negocio y registrar resultados sin confundirlos con el prototipo.</x:v>

</xml_diff>